<commit_message>
Lock CM5 power and radio interfaces before routing
</commit_message>
<xml_diff>
--- a/outputs/cm5-pin-allocation-a0/radxa_cm5_pin_allocation_a0.xlsx
+++ b/outputs/cm5-pin-allocation-a0/radxa_cm5_pin_allocation_a0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4434009b6c52444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="2" r:id="R69d61ba89f5d4827"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Map" sheetId="3" r:id="Rbf6da584f60e4dd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Allocation" sheetId="4" r:id="Rbd7c1c7691d44d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="5" r:id="R3d6b31d88f534e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Rows" sheetId="6" r:id="Rea33a2f67a0042e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1d14c325d1bb4de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="2" r:id="R8b1e480873164aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Map" sheetId="3" r:id="R6a692f90d1894a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Allocation" sheetId="4" r:id="R06ee4847aacc4fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="5" r:id="Rec82044c20eb4791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Rows" sheetId="6" r:id="Rec63f1fcad614fb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -446,7 +446,7 @@
         <x:color rgb="FF2F855A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -457,7 +457,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FF2563A6"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -479,7 +479,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -490,7 +490,7 @@
         <x:color rgb="FF2F855A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -501,7 +501,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -512,7 +512,7 @@
         <x:color rgb="FF2563A6"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -523,7 +523,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -534,7 +534,7 @@
         <x:color rgb="FF2F855A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -545,7 +545,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -556,7 +556,7 @@
         <x:color rgb="FF2563A6"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -567,7 +567,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -578,7 +578,7 @@
         <x:color rgb="FF2F855A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -589,7 +589,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -600,7 +600,7 @@
         <x:color rgb="FF2563A6"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -611,7 +611,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -622,7 +622,7 @@
         <x:color rgb="FF2F855A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -633,7 +633,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -644,7 +644,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Conflict-free interface ownership for CM5-CARRIER schematic capture | Radxa CM5 V2.21 | 2026-08-13</x:v>
+        <x:v>Conflict-free interface ownership for CM5-CARRIER schematic capture | Radxa CM5 V2.21 | 2026-08-16</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1034,12 +1034,10 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B6" s="29" t="n">
-        <x:f>COUNTIF('Assignments'!$L$5:$L$150,"LOCKED")</x:f>
-        <x:v>65</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C6" s="29" t="n">
-        <x:f>COUNTIF('Assignments'!$L$5:$L$150,"CONDITIONAL")</x:f>
-        <x:v>9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D6" s="29" t="n">
         <x:f>COUNTIF('Assignments'!$L$5:$L$150,"RESERVED")</x:f>
@@ -1050,8 +1048,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="29" t="n">
-        <x:f>COUNTIF('Conflicts'!$G$5:$G$50,"ACTION")</x:f>
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G6" s="29" t="n">
         <x:f>COUNTIF('Conflicts'!$G$5:$G$50,"BLOCKING")</x:f>
@@ -1202,7 +1199,7 @@
         <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="E16" s="69" t="str">
-        <x:v>Proceed with detailed schematic capture using these assignments. Do not begin production routing until the ACTION rows are closed, especially the monitor USB2 touch test, CM5 VCC_SYSIN tolerance check, I2C audit, PCIe sequencing review, and production-kernel pinctrl validation.</x:v>
+        <x:v>Proceed with detailed schematic capture using these assignments. Do not begin production routing until the ACTION rows are closed, especially the monitor USB2 touch test, I2C audit, PCIe sequencing review, and production-kernel pinctrl validation.</x:v>
       </x:c>
       <x:c r="F16" s="70"/>
       <x:c r="G16" s="70"/>
@@ -1228,10 +1225,10 @@
         <x:v>CM5 power setpoint</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
-        <x:v>Six VCC_SYSIN pins; final tolerance review open</x:v>
+        <x:v>Six VCC_SYSIN pins at 4.006 V; IO_5V0 supplies required HDMI-side 5 V</x:v>
       </x:c>
       <x:c r="C18" s="40" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="E18" s="72"/>
       <x:c r="F18" s="73"/>
@@ -1408,22 +1405,22 @@
         <x:v>Input</x:v>
       </x:c>
       <x:c r="K5" s="38" t="str">
-        <x:v>5 V-class input</x:v>
+        <x:v>4.006 V input</x:v>
       </x:c>
       <x:c r="L5" s="38" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M5" s="38" t="str">
-        <x:v>SYS_5V15</x:v>
+        <x:v>SYS_4V0</x:v>
       </x:c>
       <x:c r="N5" s="38" t="str">
-        <x:v>Use all six pins; release final 5.15 V setpoint only after CM5 range/tolerance review.</x:v>
+        <x:v>Use all six pins; 4.006 V target follows the Radxa CM5 carrier design note. Verify setpoint tolerance, overshoot, and connector drop.</x:v>
       </x:c>
       <x:c r="O5" s="38" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P5" s="38" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
@@ -1458,22 +1455,22 @@
         <x:v>Input</x:v>
       </x:c>
       <x:c r="K6" s="39" t="str">
-        <x:v>5 V-class input</x:v>
+        <x:v>4.006 V input</x:v>
       </x:c>
       <x:c r="L6" s="39" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M6" s="39" t="str">
-        <x:v>SYS_5V15</x:v>
+        <x:v>SYS_4V0</x:v>
       </x:c>
       <x:c r="N6" s="39" t="str">
-        <x:v>Use all six pins; release final 5.15 V setpoint only after CM5 range/tolerance review.</x:v>
+        <x:v>Use all six pins; 4.006 V target follows the Radxa CM5 carrier design note. Verify setpoint tolerance, overshoot, and connector drop.</x:v>
       </x:c>
       <x:c r="O6" s="39" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P6" s="39" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -1508,22 +1505,22 @@
         <x:v>Input</x:v>
       </x:c>
       <x:c r="K7" s="39" t="str">
-        <x:v>5 V-class input</x:v>
+        <x:v>4.006 V input</x:v>
       </x:c>
       <x:c r="L7" s="39" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M7" s="39" t="str">
-        <x:v>SYS_5V15</x:v>
+        <x:v>SYS_4V0</x:v>
       </x:c>
       <x:c r="N7" s="39" t="str">
-        <x:v>Use all six pins; release final 5.15 V setpoint only after CM5 range/tolerance review.</x:v>
+        <x:v>Use all six pins; 4.006 V target follows the Radxa CM5 carrier design note. Verify setpoint tolerance, overshoot, and connector drop.</x:v>
       </x:c>
       <x:c r="O7" s="39" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P7" s="39" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -1558,22 +1555,22 @@
         <x:v>Input</x:v>
       </x:c>
       <x:c r="K8" s="39" t="str">
-        <x:v>5 V-class input</x:v>
+        <x:v>4.006 V input</x:v>
       </x:c>
       <x:c r="L8" s="39" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M8" s="39" t="str">
-        <x:v>SYS_5V15</x:v>
+        <x:v>SYS_4V0</x:v>
       </x:c>
       <x:c r="N8" s="39" t="str">
-        <x:v>Use all six pins; release final 5.15 V setpoint only after CM5 range/tolerance review.</x:v>
+        <x:v>Use all six pins; 4.006 V target follows the Radxa CM5 carrier design note. Verify setpoint tolerance, overshoot, and connector drop.</x:v>
       </x:c>
       <x:c r="O8" s="39" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P8" s="39" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -1608,22 +1605,22 @@
         <x:v>Input</x:v>
       </x:c>
       <x:c r="K9" s="39" t="str">
-        <x:v>5 V-class input</x:v>
+        <x:v>4.006 V input</x:v>
       </x:c>
       <x:c r="L9" s="39" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M9" s="39" t="str">
-        <x:v>SYS_5V15</x:v>
+        <x:v>SYS_4V0</x:v>
       </x:c>
       <x:c r="N9" s="39" t="str">
-        <x:v>Use all six pins; release final 5.15 V setpoint only after CM5 range/tolerance review.</x:v>
+        <x:v>Use all six pins; 4.006 V target follows the Radxa CM5 carrier design note. Verify setpoint tolerance, overshoot, and connector drop.</x:v>
       </x:c>
       <x:c r="O9" s="39" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P9" s="39" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -1658,22 +1655,22 @@
         <x:v>Input</x:v>
       </x:c>
       <x:c r="K10" s="39" t="str">
-        <x:v>5 V-class input</x:v>
+        <x:v>4.006 V input</x:v>
       </x:c>
       <x:c r="L10" s="39" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M10" s="39" t="str">
-        <x:v>SYS_5V15</x:v>
+        <x:v>SYS_4V0</x:v>
       </x:c>
       <x:c r="N10" s="39" t="str">
-        <x:v>Use all six pins; release final 5.15 V setpoint only after CM5 range/tolerance review.</x:v>
+        <x:v>Use all six pins; 4.006 V target follows the Radxa CM5 carrier design note. Verify setpoint tolerance, overshoot, and connector drop.</x:v>
       </x:c>
       <x:c r="O10" s="39" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P10" s="39" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -1737,7 +1734,7 @@
         <x:v>HDMI support</x:v>
       </x:c>
       <x:c r="D12" s="39" t="str">
-        <x:v>Conditional CM5 HDMI 5 V</x:v>
+        <x:v>Required CM5 HDMI 5 V</x:v>
       </x:c>
       <x:c r="E12" s="39" t="str">
         <x:v>U13-B</x:v>
@@ -1755,25 +1752,25 @@
         <x:v>Power</x:v>
       </x:c>
       <x:c r="J12" s="39" t="str">
-        <x:v>Input / NC</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="K12" s="39" t="str">
-        <x:v>5 V</x:v>
+        <x:v>4.984 V</x:v>
       </x:c>
       <x:c r="L12" s="39" t="str">
-        <x:v>CONDITIONAL</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M12" s="39" t="str">
-        <x:v>HDMI_5V_OPTION</x:v>
+        <x:v>IO_5V0</x:v>
       </x:c>
       <x:c r="N12" s="39" t="str">
-        <x:v>Official pinout allows NC with 5 V-class VCC_SYSIN; retain a controlled DNP/link option.</x:v>
+        <x:v>Required because VCC_SYSIN is below 5 V; dedicated TPS62913 supplies CM5 pin 106.</x:v>
       </x:c>
       <x:c r="O12" s="39" t="str">
         <x:v>Radxa CM5</x:v>
       </x:c>
       <x:c r="P12" s="39" t="str">
-        <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
+        <x:v>https://dl.radxa.com/cm5/radxa_cm5_carrier_board_design_note.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -5194,7 +5191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9727138d3de0460c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bccf49067a4ab1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5724,7 +5721,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2860d7f7df4649df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R777ed66f138844c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6176,7 +6173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c7162b49c3540fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R620f2e873bac4d02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6488,22 +6485,22 @@
         <x:v>VCC_SYSIN</x:v>
       </x:c>
       <x:c r="C14" s="39" t="str">
-        <x:v>5.15 V target versus unconfirmed CM5 input tolerance</x:v>
+        <x:v>4.006 V setpoint versus CM5 input requirements</x:v>
       </x:c>
       <x:c r="D14" s="39" t="str">
-        <x:v>All six VCC_SYSIN pins</x:v>
+        <x:v>SYS_4V0 to all six VCC_SYSIN pins</x:v>
       </x:c>
       <x:c r="E14" s="39" t="str">
-        <x:v>Verify official allowed range plus setpoint, tolerance, overshoot, and connector drop.</x:v>
+        <x:v>Bench-verify setpoint tolerance, overshoot, connector drop, and full-load stability.</x:v>
       </x:c>
       <x:c r="F14" s="39" t="str">
         <x:v>HIGH</x:v>
       </x:c>
       <x:c r="G14" s="39" t="str">
-        <x:v>ACTION</x:v>
+        <x:v>CLOSED</x:v>
       </x:c>
       <x:c r="H14" s="39" t="str">
-        <x:v>Pinout identifies a 5 V-class input but does not publish the complete tolerance window.</x:v>
+        <x:v>Radxa's CM5 carrier design note recommends a 4 V VCC_SYSIN target for RK806 efficiency and performance.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
@@ -6514,22 +6511,22 @@
         <x:v>U13-B 106</x:v>
       </x:c>
       <x:c r="C15" s="39" t="str">
-        <x:v>5V_HDMI source versus no-connect</x:v>
+        <x:v>5V_HDMI source with VCC_SYSIN below 5 V</x:v>
       </x:c>
       <x:c r="D15" s="39" t="str">
-        <x:v>Controlled DNP/link option</x:v>
+        <x:v>Dedicated IO_5V0 rail</x:v>
       </x:c>
       <x:c r="E15" s="39" t="str">
-        <x:v>Resolve from final VCC_SYSIN choice and HDMI reference implementation.</x:v>
+        <x:v>Bench-verify 4.984 V at CM5 pin 106 during HDMI and USB-touch load transients.</x:v>
       </x:c>
       <x:c r="F15" s="39" t="str">
         <x:v>MEDIUM</x:v>
       </x:c>
       <x:c r="G15" s="39" t="str">
-        <x:v>ACTION</x:v>
+        <x:v>CLOSED</x:v>
       </x:c>
       <x:c r="H15" s="39" t="str">
-        <x:v>Official pinout makes this conditional on CM5 input voltage.</x:v>
+        <x:v>Radxa requires the IO board to provide 5 V on pin 106 when VCC_SYSIN is below 5 V.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -6630,7 +6627,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2856f9b9ad404b05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e1b0de5fdb43cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9535,7 +9532,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7774702243754087"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4731a6243ccb465b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Audit schematic logic against controlled datasheets
</commit_message>
<xml_diff>
--- a/outputs/cm5-pin-allocation-a0/radxa_cm5_pin_allocation_a0.xlsx
+++ b/outputs/cm5-pin-allocation-a0/radxa_cm5_pin_allocation_a0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1d14c325d1bb4de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="2" r:id="R8b1e480873164aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Map" sheetId="3" r:id="R6a692f90d1894a49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Allocation" sheetId="4" r:id="R06ee4847aacc4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="5" r:id="Rec82044c20eb4791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Rows" sheetId="6" r:id="Rec63f1fcad614fb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb2e4f04ffb544bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="2" r:id="R4c8b2938c57b4fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Map" sheetId="3" r:id="R467fa4ae301648a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Allocation" sheetId="4" r:id="R7ae2a0c227794254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="5" r:id="R9cc03862147f4e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Rows" sheetId="6" r:id="Ra28c7bf0b5a0462e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1034,14 +1034,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B6" s="29" t="n">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C6" s="29" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D6" s="29" t="n">
-        <x:f>COUNTIF('Assignments'!$L$5:$L$150,"RESERVED")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E6" s="29" t="n">
         <x:f>COUNTIF('Control Allocation'!$G$5:$G$50,"OPEN")</x:f>
@@ -2408,16 +2407,16 @@
         <x:v>3.3 V LED</x:v>
       </x:c>
       <x:c r="L25" s="39" t="str">
-        <x:v>LOCKED</x:v>
+        <x:v>RESERVED</x:v>
       </x:c>
       <x:c r="M25" s="39" t="str">
         <x:v>WAN1_LED2</x:v>
       </x:c>
       <x:c r="N25" s="39" t="str">
-        <x:v>Use the official reference LED drive method and current limits.</x:v>
+        <x:v>Selected RJ45 exposes two indicators; native LED2 is intentionally assigned no-connect in Rev A.</x:v>
       </x:c>
       <x:c r="O25" s="39" t="str">
-        <x:v>WAN1 RJ45 LEDs</x:v>
+        <x:v>Assigned no-connect on carrier</x:v>
       </x:c>
       <x:c r="P25" s="39" t="str">
         <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
@@ -2661,10 +2660,10 @@
         <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="M30" s="39" t="str">
-        <x:v>PCIE_UP_PERST_N</x:v>
+        <x:v>PCIE_UP_PERST_CMD_N</x:v>
       </x:c>
       <x:c r="N30" s="39" t="str">
-        <x:v>Host reset to PCIe switch; obey rail and reference-clock timing.</x:v>
+        <x:v>CM5 reset request is AND-gated with NET_3V3_PG and PCIE_1V0_PG before the switch receives PCIE_UP_PERST_N.</x:v>
       </x:c>
       <x:c r="O30" s="39" t="str">
         <x:v>PI7C9X2G608GP upstream</x:v>
@@ -4264,10 +4263,10 @@
         <x:v>HDMI_HEAC_N</x:v>
       </x:c>
       <x:c r="N62" s="39" t="str">
-        <x:v>Do not repurpose; decide route versus DNP with the final HDMI connector implementation.</x:v>
+        <x:v>Selected display does not use HEAC/ARC return; assigned no-connect in Rev A.</x:v>
       </x:c>
       <x:c r="O62" s="39" t="str">
-        <x:v>Lid HDMI harness</x:v>
+        <x:v>Assigned no-connect on carrier</x:v>
       </x:c>
       <x:c r="P62" s="39" t="str">
         <x:v>https://dl.radxa.com/cm5/v2210/radxa_cm5_v2210_pinout.xlsx</x:v>
@@ -5191,7 +5190,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bccf49067a4ab1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bda0850ed0541e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5284,7 +5283,7 @@
         <x:v>No external PHY</x:v>
       </x:c>
       <x:c r="H5" s="38" t="str">
-        <x:v>Direct MDI to magnetics/RJ45</x:v>
+        <x:v>Direct MDI; LED0/LED1 drive the two jack indicators and LED2 is assigned NC.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
@@ -5721,7 +5720,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R777ed66f138844c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d06ecbd09d94dd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6173,7 +6172,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R620f2e873bac4d02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaebd7a6f6d2430a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6413,7 +6412,7 @@
         <x:v>Reserved HDMI sideband</x:v>
       </x:c>
       <x:c r="E11" s="39" t="str">
-        <x:v>Choose routed versus DNP only with final HDMI connector schematic.</x:v>
+        <x:v>Route SBDP to HDMI pin 14; leave SBDN assigned NC unless a future display requires HEAC/ARC.</x:v>
       </x:c>
       <x:c r="F11" s="39" t="str">
         <x:v>LOW</x:v>
@@ -6627,7 +6626,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e1b0de5fdb43cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R385ebd9439da4fba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8498,36 +8497,16 @@
       <x:c r="D53" s="39" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="E53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="F53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="G53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="H53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="I53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="J53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="K53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="L53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="M53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="N53" s="39" t="str">
-        <x:v>414</x:v>
-      </x:c>
+      <x:c r="E53" s="39"/>
+      <x:c r="F53" s="39"/>
+      <x:c r="G53" s="39"/>
+      <x:c r="H53" s="39"/>
+      <x:c r="I53" s="39"/>
+      <x:c r="J53" s="39"/>
+      <x:c r="K53" s="39"/>
+      <x:c r="L53" s="39"/>
+      <x:c r="M53" s="39"/>
+      <x:c r="N53" s="39"/>
       <x:c r="O53" s="39" t="str"/>
       <x:c r="P53" s="39" t="str">
         <x:v>SVC-099</x:v>
@@ -9532,7 +9511,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4731a6243ccb465b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bc19310f4ef4618"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>